<commit_message>
Ahora en centro de reportes se verán diferentes datos dependiendo si eres administrador o trabajador.
</commit_message>
<xml_diff>
--- a/Registros.xlsx
+++ b/Registros.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Resumen</t>
   </si>
@@ -23,25 +23,22 @@
     <t>Horas totales</t>
   </si>
   <si>
-    <t>0h</t>
+    <t>10h</t>
   </si>
   <si>
     <t>Horas asignadas</t>
   </si>
   <si>
+    <t>8h</t>
+  </si>
+  <si>
     <t>Cumplimiento</t>
   </si>
   <si>
-    <t>NaN%</t>
+    <t>125.0%</t>
   </si>
   <si>
     <t>Proyectos activos</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>Trabajadores activos</t>
   </si>
   <si>
     <t>0</t>
@@ -89,7 +86,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -113,31 +110,23 @@
         <v>4</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s" s="0">
         <v>9</v>
-      </c>
-      <c r="B6" t="s" s="0">
-        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Tabla reportes no editable -Juanmi
</commit_message>
<xml_diff>
--- a/Registros.xlsx
+++ b/Registros.xlsx
@@ -29,19 +29,19 @@
     <t>Horas asignadas</t>
   </si>
   <si>
-    <t>8h</t>
+    <t>464h</t>
   </si>
   <si>
     <t>Cumplimiento</t>
   </si>
   <si>
-    <t>125.0%</t>
+    <t>2.1551723%</t>
   </si>
   <si>
     <t>Proyectos activos</t>
   </si>
   <si>
-    <t>0</t>
+    <t>3</t>
   </si>
 </sst>
 </file>

</xml_diff>